<commit_message>
add random + splash
</commit_message>
<xml_diff>
--- a/QBNsite/wwwroot/LoL/LolSpells.xlsx
+++ b/QBNsite/wwwroot/LoL/LolSpells.xlsx
@@ -18353,6 +18353,9 @@
       <c r="D659" s="1" t="s">
         <v>46</v>
       </c>
+      <c r="E659">
+        <v>1</v>
+      </c>
       <c r="AA659">
         <v>1</v>
       </c>
@@ -18369,9 +18372,6 @@
       </c>
       <c r="D660" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="E660">
-        <v>1</v>
       </c>
     </row>
     <row r="661" ht="14.25">
@@ -21892,7 +21892,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{A11194EB-D37D-44C8-BE7E-2B6451B75385}" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{200A5F15-C610-4BCE-93E0-5543B1504791}" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0</xm:f>
           </x14:formula1>
@@ -34133,6 +34133,9 @@
       <c r="D659" t="s">
         <v>46</v>
       </c>
+      <c r="E659">
+        <v>1</v>
+      </c>
       <c r="AA659">
         <v>1</v>
       </c>
@@ -34149,9 +34152,6 @@
       </c>
       <c r="D660" t="s">
         <v>49</v>
-      </c>
-      <c r="E660">
-        <v>1</v>
       </c>
     </row>
     <row r="661">

</xml_diff>